<commit_message>
Import product images by SKU-named files
Add an optional `image` column to the import sheet and an --images-dir
flag to the importer. Name each file after its product SKU (BH-001.png),
point the importer at the folder, and each image is uploaded to the
media library and attached to the matching product.

- `image` overrides the file name (without extension); empty falls back
  to the row's SKU, so SKU-named files need no extra data entry
- Uploads keep their file name, so media list entries read BH-001.png
- Existing uploads are reused by file name, so re-imports do not
  duplicate media
- Products that already have images are skipped unless --replace-images
- Media alt text comes from the product title (SKU as fallback), which
  is what the storefront exposes to screen readers
- Without --images-dir the behaviour is unchanged

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product-import-template.xlsx
+++ b/docs/product-import-template.xlsx
@@ -346,10 +346,20 @@
     </comment>
     <comment ref="P1" authorId="0" shapeId="0">
       <text>
+        <t>Image file name WITHOUT the extension — normally just the SKU.
+Name the file after the SKU (BH-001.png) and put it in one folder,
+then import with --images-dir=&lt;folder&gt;.
+Accepted types: .png .jpg .jpeg .webp
+Leave empty to use the SKU automatically; images are only
+imported when --images-dir is passed.</t>
+      </text>
+    </comment>
+    <comment ref="Q1" authorId="0" shapeId="0">
+      <text>
         <t>Optional country of origin, e.g. Romania.</t>
       </text>
     </comment>
-    <comment ref="Q1" authorId="0" shapeId="0">
+    <comment ref="R1" authorId="0" shapeId="0">
       <text>
         <t>Optional extra attributes as JSON, e.g. {"brand":"Balkan House"}
 Must be valid JSON or the import fails for that row.</t>
@@ -648,7 +658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q60"/>
+  <dimension ref="A1:R60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -666,8 +676,9 @@
     <col width="34" customWidth="1" min="13" max="13"/>
     <col width="34" customWidth="1" min="14" max="14"/>
     <col width="34" customWidth="1" min="15" max="15"/>
-    <col width="18" customWidth="1" min="16" max="16"/>
-    <col width="26" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="26" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -748,10 +759,15 @@
       </c>
       <c r="P1" s="2" t="inlineStr">
         <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
           <t>country_of_origin</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="R1" s="2" t="inlineStr">
         <is>
           <t>attributes</t>
         </is>
@@ -833,10 +849,15 @@
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
+          <t>BH-001</t>
+        </is>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
           <t>Romania</t>
         </is>
       </c>
-      <c r="Q2" s="3" t="inlineStr">
+      <c r="R2" s="3" t="inlineStr">
         <is>
           <t>{"brand":"Balkan House"}</t>
         </is>
@@ -860,6 +881,7 @@
       <c r="O3" s="5" t="n"/>
       <c r="P3" s="5" t="n"/>
       <c r="Q3" s="5" t="n"/>
+      <c r="R3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n"/>
@@ -879,6 +901,7 @@
       <c r="O4" s="5" t="n"/>
       <c r="P4" s="5" t="n"/>
       <c r="Q4" s="5" t="n"/>
+      <c r="R4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n"/>
@@ -898,6 +921,7 @@
       <c r="O5" s="5" t="n"/>
       <c r="P5" s="5" t="n"/>
       <c r="Q5" s="5" t="n"/>
+      <c r="R5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n"/>
@@ -917,6 +941,7 @@
       <c r="O6" s="5" t="n"/>
       <c r="P6" s="5" t="n"/>
       <c r="Q6" s="5" t="n"/>
+      <c r="R6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n"/>
@@ -936,6 +961,7 @@
       <c r="O7" s="5" t="n"/>
       <c r="P7" s="5" t="n"/>
       <c r="Q7" s="5" t="n"/>
+      <c r="R7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n"/>
@@ -955,6 +981,7 @@
       <c r="O8" s="5" t="n"/>
       <c r="P8" s="5" t="n"/>
       <c r="Q8" s="5" t="n"/>
+      <c r="R8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n"/>
@@ -974,6 +1001,7 @@
       <c r="O9" s="5" t="n"/>
       <c r="P9" s="5" t="n"/>
       <c r="Q9" s="5" t="n"/>
+      <c r="R9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n"/>
@@ -993,6 +1021,7 @@
       <c r="O10" s="5" t="n"/>
       <c r="P10" s="5" t="n"/>
       <c r="Q10" s="5" t="n"/>
+      <c r="R10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n"/>
@@ -1012,6 +1041,7 @@
       <c r="O11" s="5" t="n"/>
       <c r="P11" s="5" t="n"/>
       <c r="Q11" s="5" t="n"/>
+      <c r="R11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n"/>
@@ -1031,6 +1061,7 @@
       <c r="O12" s="5" t="n"/>
       <c r="P12" s="5" t="n"/>
       <c r="Q12" s="5" t="n"/>
+      <c r="R12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n"/>
@@ -1050,6 +1081,7 @@
       <c r="O13" s="5" t="n"/>
       <c r="P13" s="5" t="n"/>
       <c r="Q13" s="5" t="n"/>
+      <c r="R13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n"/>
@@ -1069,6 +1101,7 @@
       <c r="O14" s="5" t="n"/>
       <c r="P14" s="5" t="n"/>
       <c r="Q14" s="5" t="n"/>
+      <c r="R14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n"/>
@@ -1088,6 +1121,7 @@
       <c r="O15" s="5" t="n"/>
       <c r="P15" s="5" t="n"/>
       <c r="Q15" s="5" t="n"/>
+      <c r="R15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n"/>
@@ -1107,6 +1141,7 @@
       <c r="O16" s="5" t="n"/>
       <c r="P16" s="5" t="n"/>
       <c r="Q16" s="5" t="n"/>
+      <c r="R16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n"/>
@@ -1126,6 +1161,7 @@
       <c r="O17" s="5" t="n"/>
       <c r="P17" s="5" t="n"/>
       <c r="Q17" s="5" t="n"/>
+      <c r="R17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n"/>
@@ -1145,6 +1181,7 @@
       <c r="O18" s="5" t="n"/>
       <c r="P18" s="5" t="n"/>
       <c r="Q18" s="5" t="n"/>
+      <c r="R18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n"/>
@@ -1164,6 +1201,7 @@
       <c r="O19" s="5" t="n"/>
       <c r="P19" s="5" t="n"/>
       <c r="Q19" s="5" t="n"/>
+      <c r="R19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="n"/>
@@ -1183,6 +1221,7 @@
       <c r="O20" s="5" t="n"/>
       <c r="P20" s="5" t="n"/>
       <c r="Q20" s="5" t="n"/>
+      <c r="R20" s="5" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="n"/>
@@ -1202,6 +1241,7 @@
       <c r="O21" s="5" t="n"/>
       <c r="P21" s="5" t="n"/>
       <c r="Q21" s="5" t="n"/>
+      <c r="R21" s="5" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="n"/>
@@ -1221,6 +1261,7 @@
       <c r="O22" s="5" t="n"/>
       <c r="P22" s="5" t="n"/>
       <c r="Q22" s="5" t="n"/>
+      <c r="R22" s="5" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n"/>
@@ -1240,6 +1281,7 @@
       <c r="O23" s="5" t="n"/>
       <c r="P23" s="5" t="n"/>
       <c r="Q23" s="5" t="n"/>
+      <c r="R23" s="5" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="n"/>
@@ -1259,6 +1301,7 @@
       <c r="O24" s="5" t="n"/>
       <c r="P24" s="5" t="n"/>
       <c r="Q24" s="5" t="n"/>
+      <c r="R24" s="5" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="n"/>
@@ -1278,6 +1321,7 @@
       <c r="O25" s="5" t="n"/>
       <c r="P25" s="5" t="n"/>
       <c r="Q25" s="5" t="n"/>
+      <c r="R25" s="5" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="n"/>
@@ -1297,6 +1341,7 @@
       <c r="O26" s="5" t="n"/>
       <c r="P26" s="5" t="n"/>
       <c r="Q26" s="5" t="n"/>
+      <c r="R26" s="5" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="n"/>
@@ -1316,6 +1361,7 @@
       <c r="O27" s="5" t="n"/>
       <c r="P27" s="5" t="n"/>
       <c r="Q27" s="5" t="n"/>
+      <c r="R27" s="5" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="n"/>
@@ -1335,6 +1381,7 @@
       <c r="O28" s="5" t="n"/>
       <c r="P28" s="5" t="n"/>
       <c r="Q28" s="5" t="n"/>
+      <c r="R28" s="5" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="n"/>
@@ -1354,6 +1401,7 @@
       <c r="O29" s="5" t="n"/>
       <c r="P29" s="5" t="n"/>
       <c r="Q29" s="5" t="n"/>
+      <c r="R29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="n"/>
@@ -1373,6 +1421,7 @@
       <c r="O30" s="5" t="n"/>
       <c r="P30" s="5" t="n"/>
       <c r="Q30" s="5" t="n"/>
+      <c r="R30" s="5" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="n"/>
@@ -1392,6 +1441,7 @@
       <c r="O31" s="5" t="n"/>
       <c r="P31" s="5" t="n"/>
       <c r="Q31" s="5" t="n"/>
+      <c r="R31" s="5" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="n"/>
@@ -1411,6 +1461,7 @@
       <c r="O32" s="5" t="n"/>
       <c r="P32" s="5" t="n"/>
       <c r="Q32" s="5" t="n"/>
+      <c r="R32" s="5" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="n"/>
@@ -1430,6 +1481,7 @@
       <c r="O33" s="5" t="n"/>
       <c r="P33" s="5" t="n"/>
       <c r="Q33" s="5" t="n"/>
+      <c r="R33" s="5" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="n"/>
@@ -1449,6 +1501,7 @@
       <c r="O34" s="5" t="n"/>
       <c r="P34" s="5" t="n"/>
       <c r="Q34" s="5" t="n"/>
+      <c r="R34" s="5" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="n"/>
@@ -1468,6 +1521,7 @@
       <c r="O35" s="5" t="n"/>
       <c r="P35" s="5" t="n"/>
       <c r="Q35" s="5" t="n"/>
+      <c r="R35" s="5" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="n"/>
@@ -1487,6 +1541,7 @@
       <c r="O36" s="5" t="n"/>
       <c r="P36" s="5" t="n"/>
       <c r="Q36" s="5" t="n"/>
+      <c r="R36" s="5" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="n"/>
@@ -1506,6 +1561,7 @@
       <c r="O37" s="5" t="n"/>
       <c r="P37" s="5" t="n"/>
       <c r="Q37" s="5" t="n"/>
+      <c r="R37" s="5" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="n"/>
@@ -1525,6 +1581,7 @@
       <c r="O38" s="5" t="n"/>
       <c r="P38" s="5" t="n"/>
       <c r="Q38" s="5" t="n"/>
+      <c r="R38" s="5" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="n"/>
@@ -1544,6 +1601,7 @@
       <c r="O39" s="5" t="n"/>
       <c r="P39" s="5" t="n"/>
       <c r="Q39" s="5" t="n"/>
+      <c r="R39" s="5" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="n"/>
@@ -1563,6 +1621,7 @@
       <c r="O40" s="5" t="n"/>
       <c r="P40" s="5" t="n"/>
       <c r="Q40" s="5" t="n"/>
+      <c r="R40" s="5" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="5" t="n"/>
@@ -1582,6 +1641,7 @@
       <c r="O41" s="5" t="n"/>
       <c r="P41" s="5" t="n"/>
       <c r="Q41" s="5" t="n"/>
+      <c r="R41" s="5" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="n"/>
@@ -1601,6 +1661,7 @@
       <c r="O42" s="5" t="n"/>
       <c r="P42" s="5" t="n"/>
       <c r="Q42" s="5" t="n"/>
+      <c r="R42" s="5" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="n"/>
@@ -1620,6 +1681,7 @@
       <c r="O43" s="5" t="n"/>
       <c r="P43" s="5" t="n"/>
       <c r="Q43" s="5" t="n"/>
+      <c r="R43" s="5" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="n"/>
@@ -1639,6 +1701,7 @@
       <c r="O44" s="5" t="n"/>
       <c r="P44" s="5" t="n"/>
       <c r="Q44" s="5" t="n"/>
+      <c r="R44" s="5" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="n"/>
@@ -1658,6 +1721,7 @@
       <c r="O45" s="5" t="n"/>
       <c r="P45" s="5" t="n"/>
       <c r="Q45" s="5" t="n"/>
+      <c r="R45" s="5" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="n"/>
@@ -1677,6 +1741,7 @@
       <c r="O46" s="5" t="n"/>
       <c r="P46" s="5" t="n"/>
       <c r="Q46" s="5" t="n"/>
+      <c r="R46" s="5" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="n"/>
@@ -1696,6 +1761,7 @@
       <c r="O47" s="5" t="n"/>
       <c r="P47" s="5" t="n"/>
       <c r="Q47" s="5" t="n"/>
+      <c r="R47" s="5" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="5" t="n"/>
@@ -1715,6 +1781,7 @@
       <c r="O48" s="5" t="n"/>
       <c r="P48" s="5" t="n"/>
       <c r="Q48" s="5" t="n"/>
+      <c r="R48" s="5" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="5" t="n"/>
@@ -1734,6 +1801,7 @@
       <c r="O49" s="5" t="n"/>
       <c r="P49" s="5" t="n"/>
       <c r="Q49" s="5" t="n"/>
+      <c r="R49" s="5" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="5" t="n"/>
@@ -1753,6 +1821,7 @@
       <c r="O50" s="5" t="n"/>
       <c r="P50" s="5" t="n"/>
       <c r="Q50" s="5" t="n"/>
+      <c r="R50" s="5" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="5" t="n"/>
@@ -1772,6 +1841,7 @@
       <c r="O51" s="5" t="n"/>
       <c r="P51" s="5" t="n"/>
       <c r="Q51" s="5" t="n"/>
+      <c r="R51" s="5" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="n"/>
@@ -1791,6 +1861,7 @@
       <c r="O52" s="5" t="n"/>
       <c r="P52" s="5" t="n"/>
       <c r="Q52" s="5" t="n"/>
+      <c r="R52" s="5" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="n"/>
@@ -1810,6 +1881,7 @@
       <c r="O53" s="5" t="n"/>
       <c r="P53" s="5" t="n"/>
       <c r="Q53" s="5" t="n"/>
+      <c r="R53" s="5" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="5" t="n"/>
@@ -1829,6 +1901,7 @@
       <c r="O54" s="5" t="n"/>
       <c r="P54" s="5" t="n"/>
       <c r="Q54" s="5" t="n"/>
+      <c r="R54" s="5" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="5" t="n"/>
@@ -1848,6 +1921,7 @@
       <c r="O55" s="5" t="n"/>
       <c r="P55" s="5" t="n"/>
       <c r="Q55" s="5" t="n"/>
+      <c r="R55" s="5" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="5" t="n"/>
@@ -1867,6 +1941,7 @@
       <c r="O56" s="5" t="n"/>
       <c r="P56" s="5" t="n"/>
       <c r="Q56" s="5" t="n"/>
+      <c r="R56" s="5" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="5" t="n"/>
@@ -1886,6 +1961,7 @@
       <c r="O57" s="5" t="n"/>
       <c r="P57" s="5" t="n"/>
       <c r="Q57" s="5" t="n"/>
+      <c r="R57" s="5" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="5" t="n"/>
@@ -1905,6 +1981,7 @@
       <c r="O58" s="5" t="n"/>
       <c r="P58" s="5" t="n"/>
       <c r="Q58" s="5" t="n"/>
+      <c r="R58" s="5" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="5" t="n"/>
@@ -1924,6 +2001,7 @@
       <c r="O59" s="5" t="n"/>
       <c r="P59" s="5" t="n"/>
       <c r="Q59" s="5" t="n"/>
+      <c r="R59" s="5" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="5" t="n"/>
@@ -1943,6 +2021,7 @@
       <c r="O60" s="5" t="n"/>
       <c r="P60" s="5" t="n"/>
       <c r="Q60" s="5" t="n"/>
+      <c r="R60" s="5" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -1967,7 +2046,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2397,7 +2476,7 @@
     <row r="42">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>country_of_origin</t>
+          <t>image</t>
         </is>
       </c>
       <c r="B42" s="16" t="inlineStr">
@@ -2407,50 +2486,123 @@
       </c>
       <c r="C42" s="15" t="inlineStr">
         <is>
-          <t>Optional country of origin, e.g. Romania.</t>
+          <t>Image file name WITHOUT the extension — normally just the SKU. Name the file after the SKU (BH-001.png) and put it in one folder, then import with --images-dir=&lt;folder&gt;. Accepted types: .png .jpg .jpeg .webp Leave empty to use the SKU automatically; images are only imported when --images-dir is passed.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="13" t="inlineStr">
         <is>
+          <t>country_of_origin</t>
+        </is>
+      </c>
+      <c r="B43" s="16" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="C43" s="15" t="inlineStr">
+        <is>
+          <t>Optional country of origin, e.g. Romania.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="13" t="inlineStr">
+        <is>
           <t>attributes</t>
         </is>
       </c>
-      <c r="B43" s="16" t="inlineStr">
+      <c r="B44" s="16" t="inlineStr">
         <is>
           <t>optional</t>
         </is>
       </c>
-      <c r="C43" s="15" t="inlineStr">
+      <c r="C44" s="15" t="inlineStr">
         <is>
           <t>Optional extra attributes as JSON, e.g. {"brand":"Balkan House"} Must be valid JSON or the import fails for that row.</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="9" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
     <row r="46">
-      <c r="A46" s="8" t="inlineStr">
-        <is>
-          <t>•  Product images are NOT imported from this file. Upload them in the admin (Catalog → Media) and attach them to the product.</t>
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>Images</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>•  Header names are case-insensitive and spaces become underscores, so 'Price DKK' also works as 'price_dkk'.</t>
+          <t>1.  Name every image file after its product SKU: BH-001.png, BH-002.jpg, ...</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>2.  Put them all in one folder (any folder, e.g. product-images/).</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>3.  Leave the 'image' column empty to use the SKU automatically, or type a different file name (without extension) to override it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>4.  Import with the folder:</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    pnpm import:products -- &lt;file.xlsx&gt; --images-dir=product-images</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
+        <is>
+          <t>Each image is uploaded to the media library keeping its file name, so it appears there as BH-001.png and is easy to find by SKU. Re-running the import reuses the existing upload instead of creating duplicates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
+        <is>
+          <t>Products that already have an image are left alone; add --replace-images to overwrite them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
+        <is>
+          <t>Accepted file types: .png  .jpg  .jpeg  .webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="9" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
+        <is>
+          <t>•  Header names are case-insensitive and spaces become underscores, so 'Price DKK' also works as 'price_dkk'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
         <is>
           <t>•  Rows are validated before anything is written: if one row is invalid, the import stops and reports the row number.</t>
         </is>

</xml_diff>

<commit_message>
Remove the unused product attributes field
The free-form attributes JSON was never rendered anywhere on the
storefront and no product had any data in it (0 of 22). Its only
consumer was a one-off title backfill script, which used it as a
fallback source for missing product names.

Removed from the Products collection, the import script and the Excel
template/docs; the backfill script now derives titles from existing
locales or the SKU. The empty products.attributes column was dropped.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product-import-template.xlsx
+++ b/docs/product-import-template.xlsx
@@ -359,12 +359,6 @@
         <t>Optional country of origin, e.g. Romania.</t>
       </text>
     </comment>
-    <comment ref="R1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional extra attributes as JSON, e.g. {"brand":"Balkan House"}
-Must be valid JSON or the import fails for that row.</t>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
@@ -658,7 +652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R60"/>
+  <dimension ref="A1:Q60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -678,7 +672,6 @@
     <col width="34" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
     <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="26" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -767,11 +760,6 @@
           <t>country_of_origin</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
-        <is>
-          <t>attributes</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -855,11 +843,6 @@
       <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>Romania</t>
-        </is>
-      </c>
-      <c r="R2" s="3" t="inlineStr">
-        <is>
-          <t>{"brand":"Balkan House"}</t>
         </is>
       </c>
     </row>
@@ -881,7 +864,6 @@
       <c r="O3" s="5" t="n"/>
       <c r="P3" s="5" t="n"/>
       <c r="Q3" s="5" t="n"/>
-      <c r="R3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n"/>
@@ -901,7 +883,6 @@
       <c r="O4" s="5" t="n"/>
       <c r="P4" s="5" t="n"/>
       <c r="Q4" s="5" t="n"/>
-      <c r="R4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n"/>
@@ -921,7 +902,6 @@
       <c r="O5" s="5" t="n"/>
       <c r="P5" s="5" t="n"/>
       <c r="Q5" s="5" t="n"/>
-      <c r="R5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n"/>
@@ -941,7 +921,6 @@
       <c r="O6" s="5" t="n"/>
       <c r="P6" s="5" t="n"/>
       <c r="Q6" s="5" t="n"/>
-      <c r="R6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n"/>
@@ -961,7 +940,6 @@
       <c r="O7" s="5" t="n"/>
       <c r="P7" s="5" t="n"/>
       <c r="Q7" s="5" t="n"/>
-      <c r="R7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n"/>
@@ -981,7 +959,6 @@
       <c r="O8" s="5" t="n"/>
       <c r="P8" s="5" t="n"/>
       <c r="Q8" s="5" t="n"/>
-      <c r="R8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n"/>
@@ -1001,7 +978,6 @@
       <c r="O9" s="5" t="n"/>
       <c r="P9" s="5" t="n"/>
       <c r="Q9" s="5" t="n"/>
-      <c r="R9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n"/>
@@ -1021,7 +997,6 @@
       <c r="O10" s="5" t="n"/>
       <c r="P10" s="5" t="n"/>
       <c r="Q10" s="5" t="n"/>
-      <c r="R10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n"/>
@@ -1041,7 +1016,6 @@
       <c r="O11" s="5" t="n"/>
       <c r="P11" s="5" t="n"/>
       <c r="Q11" s="5" t="n"/>
-      <c r="R11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n"/>
@@ -1061,7 +1035,6 @@
       <c r="O12" s="5" t="n"/>
       <c r="P12" s="5" t="n"/>
       <c r="Q12" s="5" t="n"/>
-      <c r="R12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n"/>
@@ -1081,7 +1054,6 @@
       <c r="O13" s="5" t="n"/>
       <c r="P13" s="5" t="n"/>
       <c r="Q13" s="5" t="n"/>
-      <c r="R13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n"/>
@@ -1101,7 +1073,6 @@
       <c r="O14" s="5" t="n"/>
       <c r="P14" s="5" t="n"/>
       <c r="Q14" s="5" t="n"/>
-      <c r="R14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n"/>
@@ -1121,7 +1092,6 @@
       <c r="O15" s="5" t="n"/>
       <c r="P15" s="5" t="n"/>
       <c r="Q15" s="5" t="n"/>
-      <c r="R15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n"/>
@@ -1141,7 +1111,6 @@
       <c r="O16" s="5" t="n"/>
       <c r="P16" s="5" t="n"/>
       <c r="Q16" s="5" t="n"/>
-      <c r="R16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n"/>
@@ -1161,7 +1130,6 @@
       <c r="O17" s="5" t="n"/>
       <c r="P17" s="5" t="n"/>
       <c r="Q17" s="5" t="n"/>
-      <c r="R17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n"/>
@@ -1181,7 +1149,6 @@
       <c r="O18" s="5" t="n"/>
       <c r="P18" s="5" t="n"/>
       <c r="Q18" s="5" t="n"/>
-      <c r="R18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n"/>
@@ -1201,7 +1168,6 @@
       <c r="O19" s="5" t="n"/>
       <c r="P19" s="5" t="n"/>
       <c r="Q19" s="5" t="n"/>
-      <c r="R19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="n"/>
@@ -1221,7 +1187,6 @@
       <c r="O20" s="5" t="n"/>
       <c r="P20" s="5" t="n"/>
       <c r="Q20" s="5" t="n"/>
-      <c r="R20" s="5" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="n"/>
@@ -1241,7 +1206,6 @@
       <c r="O21" s="5" t="n"/>
       <c r="P21" s="5" t="n"/>
       <c r="Q21" s="5" t="n"/>
-      <c r="R21" s="5" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="n"/>
@@ -1261,7 +1225,6 @@
       <c r="O22" s="5" t="n"/>
       <c r="P22" s="5" t="n"/>
       <c r="Q22" s="5" t="n"/>
-      <c r="R22" s="5" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n"/>
@@ -1281,7 +1244,6 @@
       <c r="O23" s="5" t="n"/>
       <c r="P23" s="5" t="n"/>
       <c r="Q23" s="5" t="n"/>
-      <c r="R23" s="5" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="n"/>
@@ -1301,7 +1263,6 @@
       <c r="O24" s="5" t="n"/>
       <c r="P24" s="5" t="n"/>
       <c r="Q24" s="5" t="n"/>
-      <c r="R24" s="5" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="n"/>
@@ -1321,7 +1282,6 @@
       <c r="O25" s="5" t="n"/>
       <c r="P25" s="5" t="n"/>
       <c r="Q25" s="5" t="n"/>
-      <c r="R25" s="5" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="n"/>
@@ -1341,7 +1301,6 @@
       <c r="O26" s="5" t="n"/>
       <c r="P26" s="5" t="n"/>
       <c r="Q26" s="5" t="n"/>
-      <c r="R26" s="5" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="n"/>
@@ -1361,7 +1320,6 @@
       <c r="O27" s="5" t="n"/>
       <c r="P27" s="5" t="n"/>
       <c r="Q27" s="5" t="n"/>
-      <c r="R27" s="5" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="n"/>
@@ -1381,7 +1339,6 @@
       <c r="O28" s="5" t="n"/>
       <c r="P28" s="5" t="n"/>
       <c r="Q28" s="5" t="n"/>
-      <c r="R28" s="5" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="n"/>
@@ -1401,7 +1358,6 @@
       <c r="O29" s="5" t="n"/>
       <c r="P29" s="5" t="n"/>
       <c r="Q29" s="5" t="n"/>
-      <c r="R29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="n"/>
@@ -1421,7 +1377,6 @@
       <c r="O30" s="5" t="n"/>
       <c r="P30" s="5" t="n"/>
       <c r="Q30" s="5" t="n"/>
-      <c r="R30" s="5" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="n"/>
@@ -1441,7 +1396,6 @@
       <c r="O31" s="5" t="n"/>
       <c r="P31" s="5" t="n"/>
       <c r="Q31" s="5" t="n"/>
-      <c r="R31" s="5" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="n"/>
@@ -1461,7 +1415,6 @@
       <c r="O32" s="5" t="n"/>
       <c r="P32" s="5" t="n"/>
       <c r="Q32" s="5" t="n"/>
-      <c r="R32" s="5" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="n"/>
@@ -1481,7 +1434,6 @@
       <c r="O33" s="5" t="n"/>
       <c r="P33" s="5" t="n"/>
       <c r="Q33" s="5" t="n"/>
-      <c r="R33" s="5" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="n"/>
@@ -1501,7 +1453,6 @@
       <c r="O34" s="5" t="n"/>
       <c r="P34" s="5" t="n"/>
       <c r="Q34" s="5" t="n"/>
-      <c r="R34" s="5" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="n"/>
@@ -1521,7 +1472,6 @@
       <c r="O35" s="5" t="n"/>
       <c r="P35" s="5" t="n"/>
       <c r="Q35" s="5" t="n"/>
-      <c r="R35" s="5" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="n"/>
@@ -1541,7 +1491,6 @@
       <c r="O36" s="5" t="n"/>
       <c r="P36" s="5" t="n"/>
       <c r="Q36" s="5" t="n"/>
-      <c r="R36" s="5" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="n"/>
@@ -1561,7 +1510,6 @@
       <c r="O37" s="5" t="n"/>
       <c r="P37" s="5" t="n"/>
       <c r="Q37" s="5" t="n"/>
-      <c r="R37" s="5" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="n"/>
@@ -1581,7 +1529,6 @@
       <c r="O38" s="5" t="n"/>
       <c r="P38" s="5" t="n"/>
       <c r="Q38" s="5" t="n"/>
-      <c r="R38" s="5" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="n"/>
@@ -1601,7 +1548,6 @@
       <c r="O39" s="5" t="n"/>
       <c r="P39" s="5" t="n"/>
       <c r="Q39" s="5" t="n"/>
-      <c r="R39" s="5" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="n"/>
@@ -1621,7 +1567,6 @@
       <c r="O40" s="5" t="n"/>
       <c r="P40" s="5" t="n"/>
       <c r="Q40" s="5" t="n"/>
-      <c r="R40" s="5" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="5" t="n"/>
@@ -1641,7 +1586,6 @@
       <c r="O41" s="5" t="n"/>
       <c r="P41" s="5" t="n"/>
       <c r="Q41" s="5" t="n"/>
-      <c r="R41" s="5" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="n"/>
@@ -1661,7 +1605,6 @@
       <c r="O42" s="5" t="n"/>
       <c r="P42" s="5" t="n"/>
       <c r="Q42" s="5" t="n"/>
-      <c r="R42" s="5" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="n"/>
@@ -1681,7 +1624,6 @@
       <c r="O43" s="5" t="n"/>
       <c r="P43" s="5" t="n"/>
       <c r="Q43" s="5" t="n"/>
-      <c r="R43" s="5" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="n"/>
@@ -1701,7 +1643,6 @@
       <c r="O44" s="5" t="n"/>
       <c r="P44" s="5" t="n"/>
       <c r="Q44" s="5" t="n"/>
-      <c r="R44" s="5" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="n"/>
@@ -1721,7 +1662,6 @@
       <c r="O45" s="5" t="n"/>
       <c r="P45" s="5" t="n"/>
       <c r="Q45" s="5" t="n"/>
-      <c r="R45" s="5" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="n"/>
@@ -1741,7 +1681,6 @@
       <c r="O46" s="5" t="n"/>
       <c r="P46" s="5" t="n"/>
       <c r="Q46" s="5" t="n"/>
-      <c r="R46" s="5" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="n"/>
@@ -1761,7 +1700,6 @@
       <c r="O47" s="5" t="n"/>
       <c r="P47" s="5" t="n"/>
       <c r="Q47" s="5" t="n"/>
-      <c r="R47" s="5" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="5" t="n"/>
@@ -1781,7 +1719,6 @@
       <c r="O48" s="5" t="n"/>
       <c r="P48" s="5" t="n"/>
       <c r="Q48" s="5" t="n"/>
-      <c r="R48" s="5" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="5" t="n"/>
@@ -1801,7 +1738,6 @@
       <c r="O49" s="5" t="n"/>
       <c r="P49" s="5" t="n"/>
       <c r="Q49" s="5" t="n"/>
-      <c r="R49" s="5" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="5" t="n"/>
@@ -1821,7 +1757,6 @@
       <c r="O50" s="5" t="n"/>
       <c r="P50" s="5" t="n"/>
       <c r="Q50" s="5" t="n"/>
-      <c r="R50" s="5" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="5" t="n"/>
@@ -1841,7 +1776,6 @@
       <c r="O51" s="5" t="n"/>
       <c r="P51" s="5" t="n"/>
       <c r="Q51" s="5" t="n"/>
-      <c r="R51" s="5" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="n"/>
@@ -1861,7 +1795,6 @@
       <c r="O52" s="5" t="n"/>
       <c r="P52" s="5" t="n"/>
       <c r="Q52" s="5" t="n"/>
-      <c r="R52" s="5" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="n"/>
@@ -1881,7 +1814,6 @@
       <c r="O53" s="5" t="n"/>
       <c r="P53" s="5" t="n"/>
       <c r="Q53" s="5" t="n"/>
-      <c r="R53" s="5" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="5" t="n"/>
@@ -1901,7 +1833,6 @@
       <c r="O54" s="5" t="n"/>
       <c r="P54" s="5" t="n"/>
       <c r="Q54" s="5" t="n"/>
-      <c r="R54" s="5" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="5" t="n"/>
@@ -1921,7 +1852,6 @@
       <c r="O55" s="5" t="n"/>
       <c r="P55" s="5" t="n"/>
       <c r="Q55" s="5" t="n"/>
-      <c r="R55" s="5" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="5" t="n"/>
@@ -1941,7 +1871,6 @@
       <c r="O56" s="5" t="n"/>
       <c r="P56" s="5" t="n"/>
       <c r="Q56" s="5" t="n"/>
-      <c r="R56" s="5" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="5" t="n"/>
@@ -1961,7 +1890,6 @@
       <c r="O57" s="5" t="n"/>
       <c r="P57" s="5" t="n"/>
       <c r="Q57" s="5" t="n"/>
-      <c r="R57" s="5" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="5" t="n"/>
@@ -1981,7 +1909,6 @@
       <c r="O58" s="5" t="n"/>
       <c r="P58" s="5" t="n"/>
       <c r="Q58" s="5" t="n"/>
-      <c r="R58" s="5" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="5" t="n"/>
@@ -2001,7 +1928,6 @@
       <c r="O59" s="5" t="n"/>
       <c r="P59" s="5" t="n"/>
       <c r="Q59" s="5" t="n"/>
-      <c r="R59" s="5" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="5" t="n"/>
@@ -2021,7 +1947,6 @@
       <c r="O60" s="5" t="n"/>
       <c r="P60" s="5" t="n"/>
       <c r="Q60" s="5" t="n"/>
-      <c r="R60" s="5" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -2046,7 +1971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2507,102 +2432,85 @@
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="13" t="inlineStr">
-        <is>
-          <t>attributes</t>
-        </is>
-      </c>
-      <c r="B44" s="16" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="C44" s="15" t="inlineStr">
-        <is>
-          <t>Optional extra attributes as JSON, e.g. {"brand":"Balkan House"} Must be valid JSON or the import fails for that row.</t>
+    <row r="45">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>Images</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="9" t="inlineStr">
-        <is>
-          <t>Images</t>
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>1.  Name every image file after its product SKU: BH-001.png, BH-002.jpg, ...</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>1.  Name every image file after its product SKU: BH-001.png, BH-002.jpg, ...</t>
+          <t>2.  Put them all in one folder (any folder, e.g. product-images/).</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t>2.  Put them all in one folder (any folder, e.g. product-images/).</t>
+          <t>3.  Leave the 'image' column empty to use the SKU automatically, or type a different file name (without extension) to override it.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>3.  Leave the 'image' column empty to use the SKU automatically, or type a different file name (without extension) to override it.</t>
+          <t>4.  Import with the folder:</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t>4.  Import with the folder:</t>
+          <t xml:space="preserve">    pnpm import:products -- &lt;file.xlsx&gt; --images-dir=product-images</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">    pnpm import:products -- &lt;file.xlsx&gt; --images-dir=product-images</t>
+          <t>Each image is uploaded to the media library keeping its file name, so it appears there as BH-001.png and is easy to find by SKU. Re-running the import reuses the existing upload instead of creating duplicates.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
         <is>
-          <t>Each image is uploaded to the media library keeping its file name, so it appears there as BH-001.png and is easy to find by SKU. Re-running the import reuses the existing upload instead of creating duplicates.</t>
+          <t>Products that already have an image are left alone; add --replace-images to overwrite them.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>Products that already have an image are left alone; add --replace-images to overwrite them.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="8" t="inlineStr">
-        <is>
           <t>Accepted file types: .png  .jpg  .jpeg  .webp</t>
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" s="9" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
     <row r="56">
-      <c r="A56" s="9" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="A56" s="8" t="inlineStr">
+        <is>
+          <t>•  Header names are case-insensitive and spaces become underscores, so 'Price DKK' also works as 'price_dkk'.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
-        <is>
-          <t>•  Header names are case-insensitive and spaces become underscores, so 'Price DKK' also works as 'price_dkk'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="8" t="inlineStr">
         <is>
           <t>•  Rows are validated before anything is written: if one row is invalid, the import stops and reports the row number.</t>
         </is>

</xml_diff>